<commit_message>
Switch template research to Firecrawl and expand download links
Use Firecrawl search/scrape instead of Brave Search, add a helper
script, and refresh the valuation template catalog with additional
direct Excel downloads (DCF, LBO, comps, 3-statement).

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/fico-valuation/FICO_DCF_Valuation_Model.xlsx
+++ b/fico-valuation/FICO_DCF_Valuation_Model.xlsx
@@ -5576,7 +5576,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -5667,12 +5667,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>fcffginzu.xls (full kitchen-sink FCFF)</t>
+          <t>fcffginzu.xlsx (full kitchen-sink FCFF)</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>https://pages.stern.nyu.edu/~adamodar/pc/fcffginzu.xls</t>
+          <t>https://pages.stern.nyu.edu/~adamodar/pc/fcffginzu.xlsx</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -5772,198 +5772,198 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Corporate Finance Institute (CFI)</t>
+          <t>Babson / CFI mirror</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Free DCF Model Template</t>
+          <t>Bloomberg Practice DCF xlsx</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>https://corporatefinanceinstitute.com/resources/financial-modeling/dcf-model-template/</t>
+          <t>https://www.babson.edu/media/babson/assets/cutler-center/Bloomberg-Practice-Template.xlsx</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>3-statement linked + 5yr FCFF; email gate possible</t>
+          <t>Direct XLSX download</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CFI (direct asset)</t>
+          <t>Smartsheet</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>DCF-Valuation-Compact-Complete.xlsx</t>
+          <t>DCF Valuation xlsx</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>https://corporatefinanceinstitute.com/assets/DCF-Valuation-Compact-Complete.xlsx</t>
+          <t>https://www.smartsheet.com/sites/default/files/2020-07/IC-Discounted-Cash-Flow-Valuation-10840.xlsx</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Direct XLSX linked from CFI DCF training</t>
+          <t>Direct XLSX download</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CT Acquisitions</t>
+          <t>Corporate Finance Institute (CFI)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026 Free DCF Excel Model</t>
+          <t>Free DCF Model Template</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>https://ctacquisitions.com/dcf-template-and-excel/</t>
+          <t>https://corporatefinanceinstitute.com/resources/financial-modeling/dcf-model-template/</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>6-tab PE/IB style DCF walkthrough</t>
+          <t>3-statement linked + 5yr FCFF</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Limelight</t>
+          <t>CFI (direct asset)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Free DCF Calculator Template</t>
+          <t>DCF-Valuation-Compact-Complete.xlsx</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>https://www.golimelight.com/templates/dcf-calculator-template</t>
+          <t>https://corporatefinanceinstitute.com/assets/DCF-Valuation-Compact-Complete.xlsx</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>WACC + dual TV + scenario/sensitivity</t>
+          <t>Direct XLSX linked from CFI DCF training</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Excel Business Resource</t>
+          <t>CFI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Free DCF Model Template</t>
+          <t>Comparable company analysis template</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>https://excelbusinessresource.com/product/free-dcf-model-template-xls/</t>
+          <t>https://corporatefinanceinstitute.com/resources/financial-modeling/comparable-company-analysis-template/</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>FCFF with perpetuity + exit multiple</t>
+          <t>Trading comps</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Keene Advisors</t>
+          <t>CFI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Free DCF Model Template</t>
+          <t>3-statement case study template</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>https://www.keeneadvisors.com/free-dcf-model-template</t>
+          <t>https://corporatefinanceinstitute.com/resources/financial-modeling/case-study-3-statement-model-template/</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>3yr history + 5yr forecast DCF</t>
+          <t>Integrated model</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Macabacus</t>
+          <t>CT Acquisitions</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>DCF Model Excel Template</t>
+          <t>2026 Free DCF Excel Model</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>https://macabacus.com/excel/templates/discounted-cash-flow</t>
+          <t>https://ctacquisitions.com/dcf-template-and-excel/</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>IB-style; requires free trial for download</t>
+          <t>6-tab PE/IB style DCF walkthrough</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Macabacus</t>
+          <t>Wall Street Oasis</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Operating Model Template</t>
+          <t>DCF model template</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>https://macabacus.com/excel/templates/operating-model</t>
+          <t>https://www.wallstreetoasis.com/resources/templates/excel-financial-modeling/discounted-cash-flow-model-template</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>3-statement operating model; trial</t>
+          <t>Community template</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Macabacus</t>
+          <t>Wall Street Oasis</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>LBO Model Templates (long/short form)</t>
+          <t>LBO model template</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>https://macabacus.com/lbo-model/templates</t>
+          <t>https://www.wallstreetoasis.com/resources/templates/excel-financial-modeling/leveraged-buyout-model-template</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>LBO pack; trial</t>
+          <t>Community template</t>
         </is>
       </c>
     </row>
@@ -5975,103 +5975,257 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Free modeling resources / templates hub</t>
+          <t>LBO model lesson + template</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>https://www.wallstreetprep.com/knowledge/</t>
+          <t>https://www.wallstreetprep.com/knowledge/lbo-model/</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Articles + occasional free templates (many paid)</t>
+          <t>Free lesson + Excel</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Breaking Into Wall Street</t>
+          <t>Wall Street Prep sample</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Free financial modeling lessons / samples</t>
+          <t>LBO + DCF sample xlsx</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>https://breakingintowallstreet.com/kb/financial-modeling/</t>
+          <t>https://s3.amazonaws.com/wsp_sample_file/excel-templates/lbo-w-dcf-model-sample.xlsx</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Guides; full templates often paid</t>
+          <t>Direct sample download</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Vertex42</t>
+          <t>Exinfm</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Business valuation template (simple)</t>
+          <t>LBO DCF Model xls</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>https://www.vertex42.com/ExcelTemplates/business-valuation.html</t>
+          <t>https://exinfm.com/excel%20files/LBO_DCF_Model.xls</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Simple SME valuation workbook</t>
+          <t>Direct XLS download</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>SEC EDGAR</t>
+          <t>FE Training</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>FICO company filings (raw source)</t>
+          <t>LBO model template</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=0000814547&amp;type=10-K&amp;dateb=&amp;owner=include&amp;count=40</t>
+          <t>https://www.fe.training/free-resources/financial-modeling/lbo-model-template/</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Primary filings for FICO</t>
+          <t>Free resource</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>FE Training</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Trading comps template</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>https://www.fe.training/free-resources/investment-banking/trading-comparables-model-template/</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Free resource</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Macabacus</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>DCF Model Excel Template</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>https://macabacus.com/excel/templates/discounted-cash-flow</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>IB-style; requires free trial for download</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Macabacus</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Long-form LBO template</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>https://macabacus.com/excel/templates/lbo-model-long</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Trial</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Limelight</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Free DCF Calculator Template</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>https://www.golimelight.com/templates/dcf-calculator-template</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>WACC + dual TV + scenario/sensitivity</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Keene Advisors</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Free DCF Model Template</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>https://www.keeneadvisors.com/free-dcf-model-template</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>3yr history + 5yr forecast DCF</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Cube Software</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Free 3-statement model</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>https://www.cubesoftware.com/finance-templates/3-statement-model</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Free template</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>SEC EDGAR</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>FICO company filings (raw source)</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=0000814547&amp;type=10-K&amp;dateb=&amp;owner=include&amp;count=40</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Primary filings for FICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
           <t>SEC data API</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t>FICO companyfacts XBRL JSON</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="C31" s="4" t="inlineStr">
         <is>
           <t>https://data.sec.gov/api/xbrl/companyfacts/CIK0000814547.json</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D31" t="inlineStr">
         <is>
           <t>Machine-readable fundamentals used in this repo</t>
         </is>
@@ -6100,6 +6254,13 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId28"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>